<commit_message>
fix(dashboard): keep owners on the owner vault when agreements load first
RA-QA-08 (Major). The Documents tab chooses between the owner, tenancy and
personal views. When /me/rent-agreements answered before the /me/dashboard
aggregate that carries the owner's listings, an owner was taken for a tenant.
The tab then stayed on the tenancy view, with no renewal-relist link.

The isOwner effect now always switches to the owner view once ownership is
known, unless the user has picked a view themselves.

Also, behaviour unchanged: inlined the VaultError alias as LoadError and
removed comments that only restated the code.

Tests:
- e2e consumer/services/rent-agreement-renewal now delays /me/dashboard by
  1.5s, which makes the race deterministic. Red before the fix, 9/9 after.
- relist, doc-viewer-scheme and doc-info stay green.

Docs: e2e/COVERAGE.md renewal row; tester checklist row 312.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/Draazy-Tester-Checklist.xlsx
+++ b/docs/Draazy-Tester-Checklist.xlsx
@@ -773,7 +773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N311"/>
+  <dimension ref="A1:N312"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -20581,6 +20581,74 @@
         </is>
       </c>
       <c r="N311" s="8" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="8" t="inlineStr">
+        <is>
+          <t>311</t>
+        </is>
+      </c>
+      <c r="B312" s="8" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="C312" s="9" t="inlineStr">
+        <is>
+          <t>Renewal strip offers a relisting</t>
+        </is>
+      </c>
+      <c r="D312" s="8" t="inlineStr">
+        <is>
+          <t>As an owner with a registered rent agreement ending within 60 days, open Dashboard &gt; Documents on a slow connection.</t>
+        </is>
+      </c>
+      <c r="E312" s="8" t="inlineStr">
+        <is>
+          <t>The owner vault opens with "Renew for ₹499" and "Tenant moving out? List it again"; a tenant sees only the renewal.</t>
+        </is>
+      </c>
+      <c r="F312" s="10" t="inlineStr">
+        <is>
+          <t>/dashboard#documents</t>
+        </is>
+      </c>
+      <c r="G312" s="10" t="n"/>
+      <c r="H312" s="11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I312" s="8" t="inlineStr">
+        <is>
+          <t>QA 2026-10-16: e2e rent-agreement-renewal 9/9 incl. agreements loading before listings.</t>
+        </is>
+      </c>
+      <c r="J312" s="8" t="inlineStr">
+        <is>
+          <t>Owner; Tenant</t>
+        </is>
+      </c>
+      <c r="K312" s="8" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="L312" s="8" t="inlineStr">
+        <is>
+          <t>RA-QA-08</t>
+        </is>
+      </c>
+      <c r="M312" s="8" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="N312" s="8" t="inlineStr">
         <is>
           <t>Automated</t>
         </is>

</xml_diff>